<commit_message>
Add Sprint 1 from main
</commit_message>
<xml_diff>
--- a/Sprint_Backlog/sprint backlog.xlsx
+++ b/Sprint_Backlog/sprint backlog.xlsx
@@ -1,23 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10215"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/thanchanokkinra/Documents/PaiNamNaeWebApp/Sprint_Backlog/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{82830073-C341-C642-8BF2-D293972D2DD1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{30BD054C-987A-C244-BC69-52E65032075B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="14420" windowHeight="16140" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames>
-    <definedName name="_xlchart.v2.0" hidden="1">Sheet1!$G$36:$K$36</definedName>
-  </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
@@ -368,7 +365,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="17">
+  <cellXfs count="16">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
@@ -388,28 +385,25 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="6" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="7" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="3" xfId="0" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="ปกติ" xfId="0" builtinId="0"/>
@@ -5643,13 +5637,13 @@
       <c r="D1" s="2"/>
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
-      <c r="G1" s="7" t="s">
+      <c r="G1" s="13" t="s">
         <v>0</v>
       </c>
-      <c r="H1" s="8"/>
-      <c r="I1" s="8"/>
-      <c r="J1" s="8"/>
-      <c r="K1" s="9"/>
+      <c r="H1" s="14"/>
+      <c r="I1" s="14"/>
+      <c r="J1" s="14"/>
+      <c r="K1" s="15"/>
       <c r="L1" s="2"/>
       <c r="M1" s="1"/>
       <c r="N1" s="1"/>
@@ -7403,8 +7397,8 @@
       <c r="C39" s="1"/>
       <c r="D39" s="1"/>
       <c r="E39" s="1"/>
-      <c r="F39" s="15"/>
-      <c r="G39" s="15"/>
+      <c r="F39" s="1"/>
+      <c r="G39" s="1"/>
       <c r="H39" s="1"/>
       <c r="I39" s="1"/>
       <c r="J39" s="1"/>
@@ -7433,8 +7427,8 @@
       <c r="C40" s="1"/>
       <c r="D40" s="1"/>
       <c r="E40" s="1"/>
-      <c r="F40" s="15"/>
-      <c r="G40" s="15"/>
+      <c r="F40" s="1"/>
+      <c r="G40" s="1"/>
       <c r="H40" s="1"/>
       <c r="I40" s="1"/>
       <c r="J40" s="1"/>
@@ -7462,13 +7456,13 @@
       <c r="B41" s="1"/>
       <c r="C41" s="1"/>
       <c r="D41" s="1"/>
-      <c r="E41" s="13" t="s">
+      <c r="E41" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F41" s="16" t="s">
+      <c r="F41" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="G41" s="15"/>
+      <c r="G41" s="1"/>
       <c r="H41" s="1"/>
       <c r="I41" s="1"/>
       <c r="J41" s="1"/>
@@ -7496,13 +7490,13 @@
       <c r="B42" s="1"/>
       <c r="C42" s="1"/>
       <c r="D42" s="1"/>
-      <c r="E42" s="13">
+      <c r="E42" s="7">
         <v>1</v>
       </c>
-      <c r="F42" s="14">
+      <c r="F42" s="8">
         <v>20</v>
       </c>
-      <c r="G42" s="15"/>
+      <c r="G42" s="1"/>
       <c r="H42" s="1"/>
       <c r="I42" s="1"/>
       <c r="J42" s="1"/>
@@ -7530,13 +7524,13 @@
       <c r="B43" s="1"/>
       <c r="C43" s="1"/>
       <c r="D43" s="1"/>
-      <c r="E43" s="13">
+      <c r="E43" s="7">
         <v>2</v>
       </c>
-      <c r="F43" s="13">
+      <c r="F43" s="7">
         <v>16</v>
       </c>
-      <c r="G43" s="15"/>
+      <c r="G43" s="1"/>
       <c r="H43" s="1"/>
       <c r="I43" s="1"/>
       <c r="J43" s="1"/>
@@ -7564,13 +7558,13 @@
       <c r="B44" s="1"/>
       <c r="C44" s="1"/>
       <c r="D44" s="1"/>
-      <c r="E44" s="13">
+      <c r="E44" s="7">
         <v>3</v>
       </c>
-      <c r="F44" s="13">
+      <c r="F44" s="7">
         <v>8</v>
       </c>
-      <c r="G44" s="15"/>
+      <c r="G44" s="1"/>
       <c r="H44" s="1"/>
       <c r="I44" s="1"/>
       <c r="J44" s="1"/>
@@ -7598,10 +7592,10 @@
       <c r="B45" s="1"/>
       <c r="C45" s="1"/>
       <c r="D45" s="1"/>
-      <c r="E45" s="13">
+      <c r="E45" s="7">
         <v>4</v>
       </c>
-      <c r="F45" s="13">
+      <c r="F45" s="7">
         <v>0</v>
       </c>
       <c r="G45" s="1"/>
@@ -7632,10 +7626,10 @@
       <c r="B46" s="1"/>
       <c r="C46" s="1"/>
       <c r="D46" s="1"/>
-      <c r="E46" s="13">
+      <c r="E46" s="7">
         <v>5</v>
       </c>
-      <c r="F46" s="13">
+      <c r="F46" s="7">
         <v>0</v>
       </c>
       <c r="G46" s="1"/>
@@ -7965,10 +7959,10 @@
       <c r="B57" s="1"/>
       <c r="C57" s="1"/>
       <c r="D57" s="1"/>
-      <c r="E57" s="13" t="s">
+      <c r="E57" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F57" s="16" t="s">
+      <c r="F57" s="9" t="s">
         <v>19</v>
       </c>
       <c r="G57" s="1"/>
@@ -7999,10 +7993,10 @@
       <c r="B58" s="1"/>
       <c r="C58" s="1"/>
       <c r="D58" s="1"/>
-      <c r="E58" s="13">
+      <c r="E58" s="7">
         <v>1</v>
       </c>
-      <c r="F58" s="14">
+      <c r="F58" s="8">
         <v>17</v>
       </c>
       <c r="G58" s="1"/>
@@ -8033,10 +8027,10 @@
       <c r="B59" s="1"/>
       <c r="C59" s="1"/>
       <c r="D59" s="1"/>
-      <c r="E59" s="13">
+      <c r="E59" s="7">
         <v>2</v>
       </c>
-      <c r="F59" s="13">
+      <c r="F59" s="7">
         <v>15</v>
       </c>
       <c r="G59" s="1"/>
@@ -8067,10 +8061,10 @@
       <c r="B60" s="1"/>
       <c r="C60" s="1"/>
       <c r="D60" s="1"/>
-      <c r="E60" s="13">
+      <c r="E60" s="7">
         <v>3</v>
       </c>
-      <c r="F60" s="13">
+      <c r="F60" s="7">
         <v>6</v>
       </c>
       <c r="G60" s="1"/>
@@ -8101,10 +8095,10 @@
       <c r="B61" s="1"/>
       <c r="C61" s="1"/>
       <c r="D61" s="1"/>
-      <c r="E61" s="13">
+      <c r="E61" s="7">
         <v>4</v>
       </c>
-      <c r="F61" s="13">
+      <c r="F61" s="7">
         <v>0</v>
       </c>
       <c r="G61" s="1"/>
@@ -8135,10 +8129,10 @@
       <c r="B62" s="1"/>
       <c r="C62" s="1"/>
       <c r="D62" s="1"/>
-      <c r="E62" s="13">
+      <c r="E62" s="7">
         <v>5</v>
       </c>
-      <c r="F62" s="13">
+      <c r="F62" s="7">
         <v>0</v>
       </c>
       <c r="G62" s="1"/>
@@ -8559,10 +8553,10 @@
       <c r="B76" s="1"/>
       <c r="C76" s="1"/>
       <c r="D76" s="1"/>
-      <c r="E76" s="13" t="s">
+      <c r="E76" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F76" s="16" t="s">
+      <c r="F76" s="9" t="s">
         <v>19</v>
       </c>
       <c r="G76" s="1"/>
@@ -8593,10 +8587,10 @@
       <c r="B77" s="1"/>
       <c r="C77" s="1"/>
       <c r="D77" s="1"/>
-      <c r="E77" s="13">
+      <c r="E77" s="7">
         <v>1</v>
       </c>
-      <c r="F77" s="14">
+      <c r="F77" s="8">
         <v>17</v>
       </c>
       <c r="G77" s="1"/>
@@ -8627,10 +8621,10 @@
       <c r="B78" s="1"/>
       <c r="C78" s="1"/>
       <c r="D78" s="1"/>
-      <c r="E78" s="13">
+      <c r="E78" s="7">
         <v>2</v>
       </c>
-      <c r="F78" s="13">
+      <c r="F78" s="7">
         <v>15</v>
       </c>
       <c r="G78" s="1"/>
@@ -8661,10 +8655,10 @@
       <c r="B79" s="1"/>
       <c r="C79" s="1"/>
       <c r="D79" s="1"/>
-      <c r="E79" s="13">
+      <c r="E79" s="7">
         <v>3</v>
       </c>
-      <c r="F79" s="13">
+      <c r="F79" s="7">
         <v>6</v>
       </c>
       <c r="G79" s="1"/>
@@ -8695,10 +8689,10 @@
       <c r="B80" s="1"/>
       <c r="C80" s="1"/>
       <c r="D80" s="1"/>
-      <c r="E80" s="13">
+      <c r="E80" s="7">
         <v>4</v>
       </c>
-      <c r="F80" s="13">
+      <c r="F80" s="7">
         <v>0</v>
       </c>
       <c r="G80" s="1"/>
@@ -8729,10 +8723,10 @@
       <c r="B81" s="1"/>
       <c r="C81" s="1"/>
       <c r="D81" s="1"/>
-      <c r="E81" s="13">
+      <c r="E81" s="7">
         <v>5</v>
       </c>
-      <c r="F81" s="13">
+      <c r="F81" s="7">
         <v>0</v>
       </c>
       <c r="G81" s="1"/>
@@ -9123,10 +9117,10 @@
       <c r="B94" s="1"/>
       <c r="C94" s="1"/>
       <c r="D94" s="1"/>
-      <c r="E94" s="13" t="s">
+      <c r="E94" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F94" s="16" t="s">
+      <c r="F94" s="9" t="s">
         <v>19</v>
       </c>
       <c r="G94" s="1"/>
@@ -9157,10 +9151,10 @@
       <c r="B95" s="1"/>
       <c r="C95" s="1"/>
       <c r="D95" s="1"/>
-      <c r="E95" s="13">
+      <c r="E95" s="7">
         <v>1</v>
       </c>
-      <c r="F95" s="14">
+      <c r="F95" s="8">
         <v>14</v>
       </c>
       <c r="G95" s="1"/>
@@ -9191,10 +9185,10 @@
       <c r="B96" s="1"/>
       <c r="C96" s="1"/>
       <c r="D96" s="1"/>
-      <c r="E96" s="13">
+      <c r="E96" s="7">
         <v>2</v>
       </c>
-      <c r="F96" s="13">
+      <c r="F96" s="7">
         <v>14</v>
       </c>
       <c r="G96" s="1"/>
@@ -9225,10 +9219,10 @@
       <c r="B97" s="1"/>
       <c r="C97" s="1"/>
       <c r="D97" s="1"/>
-      <c r="E97" s="13">
+      <c r="E97" s="7">
         <v>3</v>
       </c>
-      <c r="F97" s="13">
+      <c r="F97" s="7">
         <v>8</v>
       </c>
       <c r="G97" s="1"/>
@@ -9259,10 +9253,10 @@
       <c r="B98" s="1"/>
       <c r="C98" s="1"/>
       <c r="D98" s="1"/>
-      <c r="E98" s="13">
+      <c r="E98" s="7">
         <v>4</v>
       </c>
-      <c r="F98" s="13">
+      <c r="F98" s="7">
         <v>0</v>
       </c>
       <c r="G98" s="1"/>
@@ -9293,10 +9287,10 @@
       <c r="B99" s="1"/>
       <c r="C99" s="1"/>
       <c r="D99" s="1"/>
-      <c r="E99" s="13">
+      <c r="E99" s="7">
         <v>5</v>
       </c>
-      <c r="F99" s="13">
+      <c r="F99" s="7">
         <v>0</v>
       </c>
       <c r="G99" s="1"/>
@@ -9717,10 +9711,10 @@
       <c r="B113" s="1"/>
       <c r="C113" s="1"/>
       <c r="D113" s="1"/>
-      <c r="E113" s="13" t="s">
+      <c r="E113" s="7" t="s">
         <v>47</v>
       </c>
-      <c r="F113" s="16" t="s">
+      <c r="F113" s="9" t="s">
         <v>19</v>
       </c>
       <c r="G113" s="1"/>
@@ -9751,10 +9745,10 @@
       <c r="B114" s="1"/>
       <c r="C114" s="1"/>
       <c r="D114" s="1"/>
-      <c r="E114" s="13">
+      <c r="E114" s="7">
         <v>1</v>
       </c>
-      <c r="F114" s="14">
+      <c r="F114" s="8">
         <v>14</v>
       </c>
       <c r="G114" s="1"/>
@@ -9785,10 +9779,10 @@
       <c r="B115" s="1"/>
       <c r="C115" s="1"/>
       <c r="D115" s="1"/>
-      <c r="E115" s="13">
+      <c r="E115" s="7">
         <v>2</v>
       </c>
-      <c r="F115" s="13">
+      <c r="F115" s="7">
         <v>14</v>
       </c>
       <c r="G115" s="1"/>
@@ -9819,10 +9813,10 @@
       <c r="B116" s="1"/>
       <c r="C116" s="1"/>
       <c r="D116" s="1"/>
-      <c r="E116" s="13">
+      <c r="E116" s="7">
         <v>3</v>
       </c>
-      <c r="F116" s="13">
+      <c r="F116" s="7">
         <v>3</v>
       </c>
       <c r="G116" s="1"/>
@@ -9853,10 +9847,10 @@
       <c r="B117" s="1"/>
       <c r="C117" s="1"/>
       <c r="D117" s="1"/>
-      <c r="E117" s="13">
+      <c r="E117" s="7">
         <v>4</v>
       </c>
-      <c r="F117" s="13">
+      <c r="F117" s="7">
         <v>0</v>
       </c>
       <c r="G117" s="1"/>
@@ -9887,10 +9881,10 @@
       <c r="B118" s="1"/>
       <c r="C118" s="1"/>
       <c r="D118" s="1"/>
-      <c r="E118" s="13">
+      <c r="E118" s="7">
         <v>5</v>
       </c>
-      <c r="F118" s="13">
+      <c r="F118" s="7">
         <v>0</v>
       </c>
       <c r="G118" s="1"/>

</xml_diff>